<commit_message>
feat(programming): combine COD session
Agent: codcombine
</commit_message>
<xml_diff>
--- a/docs/CONDITIONING_TEMPLATES_FINAL_2026-07-25.xlsx
+++ b/docs/CONDITIONING_TEMPLATES_FINAL_2026-07-25.xlsx
@@ -2,20 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture &amp; Rules" sheetId="1" r:id="R7a37f87075c7407f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="2" r:id="R327c39fe211a4810"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceleration" sheetId="3" r:id="Rcc89c6e2c9b84985"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top End Speed" sheetId="4" r:id="R1598129cc57a41fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repeat Sprint" sheetId="5" r:id="Rdc9bc2cf5aa24ab1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change of Direction-Decel" sheetId="6" r:id="R0e23a6465513456b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anaerobic" sheetId="7" r:id="R4d242303ad7f43d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aerobic Power" sheetId="8" r:id="R8ffc1b60b0614d7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aerobic Capacity" sheetId="9" r:id="R4a6706444d9e46b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flush" sheetId="10" r:id="R142fca3677c74ff1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="11" r:id="Ra20e0637eae942b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Questions (Sam)" sheetId="12" r:id="R5bf710ec4d71468b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skim List" sheetId="13" r:id="R791d019801aa4607"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="V3 Rulings" sheetId="14" r:id="R588575a4c751470a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture &amp; Rules" sheetId="1" r:id="R81b17f5abb044d35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="2" r:id="Reef794f5301e456a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceleration" sheetId="3" r:id="R9f7d66ae5bc24fd5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top End Speed" sheetId="4" r:id="R7b8443ffb5e14697"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repeat Sprint" sheetId="5" r:id="Raab62ca624024e34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change of Direction-Decel" sheetId="6" r:id="R59b23763cfc941b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anaerobic" sheetId="7" r:id="R20d42b6fea604444"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aerobic Power" sheetId="8" r:id="Rb03e1bc7b2ad4eb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aerobic Capacity" sheetId="9" r:id="Rf8c17916c6874445"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flush" sheetId="10" r:id="R3a43b7fb80114c39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change Log" sheetId="11" r:id="R614c16d0ca814c35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Questions (Sam)" sheetId="12" r:id="Rb189679ba78f42ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skim List" sheetId="13" r:id="R8194b813a02d429f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="V3 Rulings" sheetId="14" r:id="R5cca0ea5cad948a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COD Session Sections" sheetId="15" r:id="Rc7bd147999bd4641"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -26,7 +27,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="6">
+  <x:fonts count="7">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -52,8 +53,14 @@
       <x:b/>
       <x:color rgb="FF9C0006"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Calibri"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -68,6 +75,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F3864"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -91,7 +103,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="11">
+  <x:cellXfs count="17">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
@@ -121,6 +133,16 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -196,6 +218,22 @@
     </x:indexedColors>
   </x:colors>
 </x:styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CodSessionSectionsTable" displayName="CodSessionSectionsTable" ref="A1:H4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="8">
+    <x:tableColumn id="1" name="Session"/>
+    <x:tableColumn id="2" name="Order"/>
+    <x:tableColumn id="3" name="Section"/>
+    <x:tableColumn id="4" name="Work"/>
+    <x:tableColumn id="5" name="Recovery"/>
+    <x:tableColumn id="6" name="Amount"/>
+    <x:tableColumn id="7" name="Effort"/>
+    <x:tableColumn id="8" name="Cue"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -418,514 +456,342 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="1" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">The Conditioning Templates — FINAL (2026-07-25)</x:t>
-        </x:is>
+      <x:c r="A1" s="1" t="str">
+        <x:v>The Conditioning Templates — FINAL (2026-07-25)</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">AUTHORED FINAL — Sam sign-off 2026-07-25/27. SOURCE OF TRUTH for the conditioning build; changes require Sam.</x:t>
-        </x:is>
+      <x:c r="A2" s="2" t="str">
+        <x:v>AUTHORED FINAL — Sam sign-off 2026-07-25/27. SOURCE OF TRUTH for the conditioning build; changes require Sam.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="A3" s="3"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">All twenty-one rulings applied. 55 templates, zero flags, empty Skim List.</x:t>
-        </x:is>
+      <x:c r="A4" s="3" t="str">
+        <x:v>All twenty-one rulings applied. 52 templates, zero flags, empty Skim List.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="A5" s="3"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">WHAT GOVERNS THIS SHEET</x:t>
-        </x:is>
+      <x:c r="A6" s="2" t="str">
+        <x:v>WHAT GOVERNS THIS SHEET</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">CONDITIONING_FRAMEWORK_SAM_2026-07-25.md (Sam's authored physiology) outranks every earlier draft sorting. V2's base state was conditioning_templates_sam_state_2026-07-25.json. V3 applies Sam's five rulings on the V2 open questions — listed on the 'V3 Rulings' tab, and named at every row they touch.</x:t>
-        </x:is>
+      <x:c r="A7" s="3" t="str">
+        <x:v>CONDITIONING_FRAMEWORK_SAM_2026-07-25.md (Sam's authored physiology) outranks every earlier draft sorting. V2's base state was conditioning_templates_sam_state_2026-07-25.json. V3 applies Sam's five rulings on the V2 open questions — listed on the 'V3 Rulings' tab, and named at every row they touch.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="A8" s="3"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">*** THE CLASSIFICATION LAW (Sam, V3-final) ***</x:t>
-        </x:is>
+      <x:c r="A9" s="2" t="str">
+        <x:v>*** THE CLASSIFICATION LAW (Sam, V3-final) ***</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">INTENSITY CLASSIFIES. W:R IS ONLY A PROPERTY.</x:t>
-        </x:is>
+      <x:c r="A10" s="2" t="str">
+        <x:v>INTENSITY CLASSIFIES. W:R IS ONLY A PROPERTY.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">A session belongs to the quality its INTENSITY says it belongs to. Its work-to-rest ratio describes the session; it does not decide which quality the session is. A W:R outside a quality's tabled band is therefore a property of that session, not a misfiling and not an error. Effort length reads the same way. This law governs every row in this sheet and retires the whole class of 'ratio outside band' flags: after it, 9 flags cleared at once (4 tempo rows, 3 protocol rows, and the two short-intermittent aerobic-power rows), leaving only genuinely INFERRED numbers to review.</x:t>
-        </x:is>
+      <x:c r="A11" s="3" t="str">
+        <x:v>A session belongs to the quality its INTENSITY says it belongs to. Its work-to-rest ratio describes the session; it does not decide which quality the session is. A W:R outside a quality's tabled band is therefore a property of that session, not a misfiling and not an error. Effort length reads the same way. This law governs every row in this sheet and retires the whole class of 'ratio outside band' flags: after it, 9 flags cleared at once (4 tempo rows, 3 protocol rows, and the two short-intermittent aerobic-power rows), leaving only genuinely INFERRED numbers to review.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="A12" s="3"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">THE SHORT-INTERMITTENT MAS RULE (Sam, FINAL ruling 1)</x:t>
-        </x:is>
+      <x:c r="A13" s="2" t="str">
+        <x:v>THE SHORT-INTERMITTENT MAS RULE (Sam, FINAL ruling 1)</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">High-%MAS short reps (the 15:15 class) build AEROBIC POWER provided the set stays contained: SET / BLOCK &lt;= ~4–5 MIN, with rest between blocks. A short-rep session that runs unbroken past that is no longer aerobic-power work. Carried as the SET LENGTH property on MAS 15:15, 30:30 Hard Intermittent and Erg EMOM — the last two were RESTRUCTURED into blocks to comply.</x:t>
-        </x:is>
+      <x:c r="A14" s="3" t="str">
+        <x:v>High-%MAS short reps (the 15:15 class) build AEROBIC POWER provided the set stays contained: SET / BLOCK &lt;= ~4–5 MIN, with rest between blocks. A short-rep session that runs unbroken past that is no longer aerobic-power work. Carried as the SET LENGTH property on MAS 15:15, 30:30 Hard Intermittent and Erg EMOM — the last two were RESTRUCTURED into blocks to comply.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="A15" s="3"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">TEMPLATE PROPERTIES (machine-readable, in the Properties column)</x:t>
-        </x:is>
+      <x:c r="A16" s="2" t="str">
+        <x:v>TEMPLATE PROPERTIES (machine-readable, in the Properties column)</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SET LENGTH &lt;= 4-5 min — short-intermittent MAS rule (ruling 1).</x:t>
-        </x:is>
+      <x:c r="A17" s="3" t="str">
+        <x:v>SET LENGTH &lt;= 4-5 min — short-intermittent MAS rule (ruling 1).</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">FINISHER ROLE ONLY · ERG ONLY · single set — Tabata Finisher (ruling 6). Never prescribed as the session itself; one set, 4 min max, ergs only.</x:t>
-        </x:is>
+      <x:c r="A18" s="3" t="str">
+        <x:v>FINISHER ROLE ONLY · ERG ONLY · single set — Tabata Finisher (ruling 6). Never prescribed as the session itself; one set, 4 min max, ergs only.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">FALLBACK ONLY (no-equipment athletes) — Bodyweight Circuit (ruling 9). Never in-season or pre-season.</x:t>
-        </x:is>
+      <x:c r="A19" s="3" t="str">
+        <x:v>FALLBACK ONLY (no-equipment athletes) — Bodyweight Circuit (ruling 9). Never in-season or pre-season.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">AVAILABILITY GATE: no-team-training weeks only · LOW selection priority — the whole Change of Direction-Decel row (ruling 5). Prescribed only in weeks with NO team training (late off-season, Christmas break), and last in line when something must be cut.</x:t>
-        </x:is>
+      <x:c r="A20" s="3" t="str">
+        <x:v>AVAILABILITY GATE: no-team-training weeks only · LOW selection priority — the one combined Change of Direction session. Prescribe only in weeks with NO team training (late off-season, Christmas break), and last in line when something must be cut.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">MID-SESSION MIXING ALLOWED (flush-only) — the three Flush Intervals rows (ruling 5 of the V3 set).</x:t>
-        </x:is>
+      <x:c r="A21" s="3" t="str">
+        <x:v>MID-SESSION MIXING ALLOWED (flush-only) — the three Flush Intervals rows (ruling 5 of the V3 set).</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="A22" s="3"/>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SAM'S RULINGS (2026-07-25) — all applied</x:t>
-        </x:is>
+      <x:c r="A23" s="2" t="str">
+        <x:v>SAM'S RULINGS (2026-07-25) — all applied</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">1. SPRINT-FAMILY EXEMPTION from the 1:12 alactic ceiling: full recovery at 1:10–1:15+ is allowed. 9 ⚑ RATIO flags cleared (5 Acceleration, 4 Top End Speed).</x:t>
-        </x:is>
+      <x:c r="A24" s="3" t="str">
+        <x:v>1. SPRINT-FAMILY EXEMPTION from the 1:12 alactic ceiling: full recovery at 1:10–1:15+ is allowed. 9 ⚑ RATIO flags cleared (5 Acceleration, 4 Top End Speed).</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2. 150–200 m Hard Repeats: STRUCTURE changed to 'departing every 2:00' (not just relabelled). True ratio ~1:3–1:4, in band. Flag cleared.</x:t>
-        </x:is>
+      <x:c r="A25" s="3" t="str">
+        <x:v>2. 150–200 m Hard Repeats: STRUCTURE changed to 'departing every 2:00' (not just relabelled). True ratio ~1:3–1:4, in band. Flag cleared.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">3. Extensive Tempo: session UNCHANGED, ratio label corrected to ~1:2 (the framework's '~2:1' was a labelling error).</x:t>
-        </x:is>
+      <x:c r="A26" s="3" t="str">
+        <x:v>3. Extensive Tempo: session UNCHANGED, ratio label corrected to ~1:2 (the framework's '~2:1' was a labelling error).</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">4. Repeated Jumps (5×3 broad jumps) DELETED entirely — jump work lives in the POWER SYSTEM only, not in conditioning. Bike power 8×6 s becomes 'Air Bike Accelerations' in the Acceleration tab. This resolves the V2 taxonomy flag as OPTION A: an alactic non-run variant lives in Acceleration via Modality Notes; no Anaerobic Power tab is added.</x:t>
-        </x:is>
+      <x:c r="A27" s="3" t="str">
+        <x:v>4. Repeated Jumps (5×3 broad jumps) DELETED entirely — jump work lives in the POWER SYSTEM only, not in conditioning. Bike power 8×6 s becomes 'Air Bike Accelerations' in the Acceleration tab. This resolves the V2 taxonomy flag as OPTION A: an alactic non-run variant lives in Acceleration via Modality Notes; no Anaerobic Power tab is added.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">5. FLUSH CONFIRMED at 7 rows: the 4 consolidated sessions (draft markers removed) plus 3 Sam-authored interval flushes (30:30, 1:1, 2:1), all at 3–4/10 MAX, any modality, mid-session mixing allowed.</x:t>
-        </x:is>
+      <x:c r="A28" s="3" t="str">
+        <x:v>5. FLUSH CONFIRMED at 7 rows: the 4 consolidated sessions (draft markers removed) plus 3 Sam-authored interval flushes (30:30, 1:1, 2:1), all at 3–4/10 MAX, any modality, mid-session mixing allowed.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">6. V3-FINAL — INTENSITY CLASSIFIES, W:R IS ONLY A PROPERTY (the law above). The tempo cluster (30:30 controlled, 1 min on/1 min, 2 min on/1 min, extensive tempo) sits where its intensity says; all four flags cleared, along with every other ratio/effort-length flag on a non-inferred row.</x:t>
-        </x:is>
+      <x:c r="A29" s="3" t="str">
+        <x:v>6. V3-FINAL — INTENSITY CLASSIFIES, W:R IS ONLY A PROPERTY (the law above). The tempo cluster (30:30 controlled, 1 min on/1 min, 2 min on/1 min, extensive tempo) sits where its intensity says; all four flags cleared, along with every other ratio/effort-length flag on a non-inferred row.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">7. V3-FINAL — 400 m Repeats depart every 3:00 (structure, not label): rest is the 3:00 remainder (≈100–105 s), ~1:1-ish aerobic power. Flag cleared.</x:t>
-        </x:is>
+      <x:c r="A30" s="3" t="str">
+        <x:v>7. V3-FINAL — 400 m Repeats depart every 3:00 (structure, not label): rest is the 3:00 remainder (≈100–105 s), ~1:1-ish aerobic power. Flag cleared.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">8. V3-FINAL — Deceleration and Landing Work STAYS in Change of Direction-Decel: landing mechanics, not jump training (the deleted repeated-jumps session was jump training).</x:t>
-        </x:is>
+      <x:c r="A31" s="3" t="str">
+        <x:v>8. SUPERSEDED 2026-09-02 — Deceleration and Landing Work was removed when the COD catalogue became one combined Change of Direction session.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">9. FINAL — short-intermittent aerobic power confirmed with the set-length rule above (MAS 15:15, 30:30 Hard Intermittent, Erg EMOM; the Erg EMOM 40 s/20 s split is confirmed).</x:t>
-        </x:is>
+      <x:c r="A32" s="3" t="str">
+        <x:v>9. FINAL — short-intermittent aerobic power confirmed with the set-length rule above (MAS 15:15, 30:30 Hard Intermittent, Erg EMOM; the Erg EMOM 40 s/20 s split is confirmed).</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">10. FINAL — 30 m Acceleration Reps raised to 95–100% (technique work lives in warm-ups).</x:t>
-        </x:is>
+      <x:c r="A33" s="3" t="str">
+        <x:v>10. FINAL — 30 m Acceleration Reps raised to 95–100% (technique work lives in warm-ups).</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
-      <x:c r="A34" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">11. FINAL — Resisted Band Acceleration BINNED.</x:t>
-        </x:is>
+      <x:c r="A34" s="3" t="str">
+        <x:v>11. FINAL — Resisted Band Acceleration BINNED.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
-      <x:c r="A35" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">12. FINAL — Inverse Tabata restructured to 10 s / 30 s and renamed '10 s Repeat Efforts'.</x:t>
-        </x:is>
+      <x:c r="A35" s="3" t="str">
+        <x:v>12. FINAL — Inverse Tabata restructured to 10 s / 30 s and renamed '10 s Repeat Efforts'.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">13. FINAL — COD keeps 4 rows (Up-Back Shuttle, Low-Intensity Decel, Decel and Landing, 45-Degree Cut); Short COD Circuit and COD Finisher binned; the whole row gains the availability gate; doses approved.</x:t>
-        </x:is>
+      <x:c r="A36" s="3" t="str">
+        <x:v>13. UPDATED 2026-09-02 — COD is one selectable Change of Direction session: Speed warm-up, Low-Intensity Deceleration Drills, 45-Degree Cut Reps, then Up-Back Shuttle. The former individual templates and Deceleration and Landing Work are not separate choices.</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
-      <x:c r="A37" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">14. FINAL — Tabata kept as Tabata Finisher: erg-only, finisher-role-only, single set, 4 min max.</x:t>
-        </x:is>
+      <x:c r="A37" s="3" t="str">
+        <x:v>14. FINAL — Tabata kept as Tabata Finisher: erg-only, finisher-role-only, single set, 4 min max.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
-      <x:c r="A38" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">15. FINAL — 45 s Hard Repeats: descending-rest variant dropped, base row stands.</x:t>
-        </x:is>
+      <x:c r="A38" s="3" t="str">
+        <x:v>15. FINAL — 45 s Hard Repeats: descending-rest variant dropped, base row stands.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
-      <x:c r="A39" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">16. FINAL — 60-90 s Max Sustained capped at 60 s.</x:t>
-        </x:is>
+      <x:c r="A39" s="3" t="str">
+        <x:v>16. FINAL — 60-90 s Max Sustained capped at 60 s.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
-      <x:c r="A40" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">17. FINAL — Bodyweight Circuit kept as fallback-only.</x:t>
-        </x:is>
+      <x:c r="A40" s="3" t="str">
+        <x:v>17. FINAL — Bodyweight Circuit kept as fallback-only.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
-      <x:c r="A41" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="A41" s="3"/>
     </x:row>
     <x:row r="42">
-      <x:c r="A42" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">THE GOVERNING TABLE (Sam's) — every row is checked against it</x:t>
-        </x:is>
+      <x:c r="A42" s="2" t="str">
+        <x:v>THE GOVERNING TABLE (Sam's) — every row is checked against it</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
-      <x:c r="A43" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Anaerobic power (alactic)          effort 3–10 s      W:R 1:6–1:12*     max speed and explosiveness</x:t>
-        </x:is>
+      <x:c r="A43" s="3" t="str">
+        <x:v>Anaerobic power (alactic)          effort 3–10 s      W:R 1:6–1:12*     max speed and explosiveness</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
-      <x:c r="A44" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Repeated-sprint ability            effort 4–10 s      W:R 1:3–1:5       repeat high-speed efforts</x:t>
-        </x:is>
+      <x:c r="A44" s="3" t="str">
+        <x:v>Repeated-sprint ability            effort 4–10 s      W:R 1:3–1:5       repeat high-speed efforts</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
-      <x:c r="A45" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Anaerobic capacity (glycolytic)    effort 15–60 s     W:R 1:2–1:5       sustain hard work through fatigue</x:t>
-        </x:is>
+      <x:c r="A45" s="3" t="str">
+        <x:v>Anaerobic capacity (glycolytic)    effort 15–60 s     W:R 1:2–1:5       sustain hard work through fatigue</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
-      <x:c r="A46" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Aerobic power                      effort 1–5 min     W:R 1:1–2:1       high aerobic output</x:t>
-        </x:is>
+      <x:c r="A46" s="3" t="str">
+        <x:v>Aerobic power                      effort 1–5 min     W:R 1:1–2:1       high aerobic output</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
-      <x:c r="A47" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Aerobic capacity                   longer/continuous     W:R 3:1–continuous    total sustainable aerobic work</x:t>
-        </x:is>
+      <x:c r="A47" s="3" t="str">
+        <x:v>Aerobic capacity                   longer/continuous     W:R 3:1–continuous    total sustainable aerobic work</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
-      <x:c r="A48" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">* SPRINT-FAMILY EXEMPTION (ruling 1): for alactic sprint work the 1:12 ceiling is NOT binding — full recovery at 1:10–1:15+ is allowed and is not flagged. The 1:6 floor still holds.</x:t>
-        </x:is>
+      <x:c r="A48" s="3" t="str">
+        <x:v>* SPRINT-FAMILY EXEMPTION (ruling 1): for alactic sprint work the 1:12 ceiling is NOT binding — full recovery at 1:10–1:15+ is allowed and is not flagged. The 1:6 floor still holds.</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
-      <x:c r="A49" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="A49" s="3"/>
     </x:row>
     <x:row r="50">
-      <x:c r="A50" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">WHICH TAB MAPS TO WHICH FRAMEWORK QUALITY</x:t>
-        </x:is>
+      <x:c r="A50" s="2" t="str">
+        <x:v>WHICH TAB MAPS TO WHICH FRAMEWORK QUALITY</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
-      <x:c r="A51" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Acceleration + Top End Speed  -&gt;  anaerobic power (alactic). Acceleration now also holds the one non-run alactic row, Air Bike Accelerations (ruling 4).</x:t>
-        </x:is>
+      <x:c r="A51" s="3" t="str">
+        <x:v>Acceleration + Top End Speed  -&gt;  anaerobic power (alactic). Acceleration now also holds the one non-run alactic row, Air Bike Accelerations (ruling 4).</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
-      <x:c r="A52" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Repeat Sprint                 -&gt;  repeated-sprint ability</x:t>
-        </x:is>
+      <x:c r="A52" s="3" t="str">
+        <x:v>Repeat Sprint                 -&gt;  repeated-sprint ability</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
-      <x:c r="A53" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Anaerobic                     -&gt;  anaerobic capacity (glycolytic). GRIND IS DISSOLVED IN HERE (Sam's ruling).</x:t>
-        </x:is>
+      <x:c r="A53" s="3" t="str">
+        <x:v>Anaerobic                     -&gt;  anaerobic capacity (glycolytic). GRIND IS DISSOLVED IN HERE (Sam's ruling).</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
-      <x:c r="A54" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Aerobic Power                 -&gt;  aerobic power</x:t>
-        </x:is>
+      <x:c r="A54" s="3" t="str">
+        <x:v>Aerobic Power                 -&gt;  aerobic power</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
-      <x:c r="A55" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Aerobic Capacity              -&gt;  aerobic capacity</x:t>
-        </x:is>
+      <x:c r="A55" s="3" t="str">
+        <x:v>Aerobic Capacity              -&gt;  aerobic capacity</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
-      <x:c r="A56" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Change of Direction/Decel     -&gt;  NO framework row (mechanics quality) — unbanded, see Open Q6</x:t>
-        </x:is>
+      <x:c r="A56" s="3" t="str">
+        <x:v>Change of Direction/Decel -&gt; NO framework row (mechanics quality) — one combined Run-only session, unbanded.</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
-      <x:c r="A57" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Flush                         -&gt;  NO framework row (recovery, not a trained quality). 7 rows, confirmed.</x:t>
-        </x:is>
+      <x:c r="A57" s="3" t="str">
+        <x:v>Flush                         -&gt;  NO framework row (recovery, not a trained quality). 7 rows, confirmed.</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
-      <x:c r="A58" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="A58" s="3"/>
     </x:row>
     <x:row r="59">
-      <x:c r="A59" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">THE SCHEMA (every row carries all six)</x:t>
-        </x:is>
+      <x:c r="A59" s="2" t="str">
+        <x:v>THE SCHEMA (every row carries all six)</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
-      <x:c r="A60" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Work period — Rest period — Sets/rounds (reps) — Intensity (framework language: %MAS / %HRmax / effort words) — W:R ratio — Total session time. Total session time = work + rest only (add warm-up and cool-down on top).</x:t>
-        </x:is>
+      <x:c r="A60" s="3" t="str">
+        <x:v>Work period — Rest period — Sets/rounds (reps) — Intensity (framework language: %MAS / %HRmax / effort words) — W:R ratio — Total session time. Total session time = work + rest only (add warm-up and cool-down on top).</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
-      <x:c r="A61" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="A61" s="3"/>
     </x:row>
     <x:row r="62">
-      <x:c r="A62" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">D14 — THE RENDERING LAYER FOR %MAS RUN WORK</x:t>
-        </x:is>
+      <x:c r="A62" s="2" t="str">
+        <x:v>D14 — THE RENDERING LAYER FOR %MAS RUN WORK</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
-      <x:c r="A63" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Every %MAS intensity in this sheet renders per-athlete through D14 (PROGRAMMING_DESIGN_SESSION_2026-07-23.md, 'MAS via 2 km time trial', Sam 2026-07-25): onboarding gains a 2 km TT screen (skippable — MAS then defaults by experience level so every MAS session still renders); MAS is stored on-device; %MAS intensities become per-athlete paces and rep distances; a 2 km TT is re-prescribed as a real aerobic-power session every ~6–8 weeks to recalibrate. So '90–100% MAS' in these rows is a rendering instruction, not a fixed pace.</x:t>
-        </x:is>
+      <x:c r="A63" s="3" t="str">
+        <x:v>Every %MAS intensity in this sheet renders per-athlete through D14 (PROGRAMMING_DESIGN_SESSION_2026-07-23.md, 'MAS via 2 km time trial', Sam 2026-07-25): onboarding gains a 2 km TT screen (skippable — MAS then defaults by experience level so every MAS session still renders); MAS is stored on-device; %MAS intensities become per-athlete paces and rep distances; a 2 km TT is re-prescribed as a real aerobic-power session every ~6–8 weeks to recalibrate. So '90–100% MAS' in these rows is a rendering instruction, not a fixed pace.</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
-      <x:c r="A64" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="A64" s="3"/>
     </x:row>
     <x:row r="65">
-      <x:c r="A65" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">THE ⚑ FLAGS</x:t>
-        </x:is>
+      <x:c r="A65" s="2" t="str">
+        <x:v>THE ⚑ FLAGS</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
-      <x:c r="A66" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">NO FLAGS REMAIN. The classification law retired ⚑ RATIO and ⚑ BAND as a class; Sam's final skim rulings cleared the last ⚑ INFERRED doses by approving, restructuring or binning every one of them. The Skim List tab is empty. Any future template that arrives without a Sam-authored or framework dose gets a ⚑ INFERRED mark and lands there.</x:t>
-        </x:is>
+      <x:c r="A66" s="3" t="str">
+        <x:v>NO FLAGS REMAIN. The classification law retired ⚑ RATIO and ⚑ BAND as a class; Sam's final skim rulings cleared the last ⚑ INFERRED doses by approving, restructuring or binning every one of them. The Skim List tab is empty. Any future template that arrives without a Sam-authored or framework dose gets a ⚑ INFERRED mark and lands there.</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
-      <x:c r="A67" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="A67" s="3"/>
     </x:row>
     <x:row r="68">
-      <x:c r="A68" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">EFFORT-LENGTH ASSUMPTIONS (used to compute work periods and W:R from distance rows)</x:t>
-        </x:is>
+      <x:c r="A68" s="2" t="str">
+        <x:v>EFFORT-LENGTH ASSUMPTIONS (used to compute work periods and W:R from distance rows)</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
-      <x:c r="A69" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">10 m ≈ 2 s  ·  20 m ≈ 3 s  ·  20 m shuttle (2×10 m) ≈ 4 s  ·  30 m ≈ 4.5 s  ·  40–60 m ≈ 6–8 s  ·  20+20 fly ≈ 6 s  ·  30+30 fly ≈ 8 s</x:t>
-        </x:is>
+      <x:c r="A69" s="3" t="str">
+        <x:v>10 m ≈ 2 s  ·  20 m ≈ 3 s  ·  20 m shuttle (2×10 m) ≈ 4 s  ·  30 m ≈ 4.5 s  ·  40–60 m ≈ 6–8 s  ·  20+20 fly ≈ 6 s  ·  30+30 fly ≈ 8 s</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
-      <x:c r="A70" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">100 m @65–75% ≈ 16 s  ·  150 m ≈ 22 s  ·  200 m ≈ 30 s  ·  400 m ≈ 75–80 s  ·  1 km ≈ 3.5–4 min. Walk-back/walk-down recovery is timed, not assumed instant.</x:t>
-        </x:is>
+      <x:c r="A70" s="3" t="str">
+        <x:v>100 m @65–75% ≈ 16 s  ·  150 m ≈ 22 s  ·  200 m ≈ 30 s  ·  400 m ≈ 75–80 s  ·  1 km ≈ 3.5–4 min. Walk-back/walk-down recovery is timed, not assumed instant.</x:v>
       </x:c>
     </x:row>
     <x:row r="71">
-      <x:c r="A71" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="A71" s="3"/>
     </x:row>
     <x:row r="72">
-      <x:c r="A72" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">STANDING RENDERING RULES</x:t>
-        </x:is>
+      <x:c r="A72" s="2" t="str">
+        <x:v>STANDING RENDERING RULES</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
-      <x:c r="A73" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">1. TIME-FIRST. Distance is allowed for short/speed work and mid-length reps; calories for EMOM-class erg work.</x:t>
-        </x:is>
+      <x:c r="A73" s="3" t="str">
+        <x:v>1. TIME-FIRST. Distance is allowed for short/speed work and mid-length reps; calories for EMOM-class erg work.</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
@@ -944,45 +810,31 @@
       </x:c>
     </x:row>
     <x:row r="77">
-      <x:c r="A77" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">5. NO SLEDS anywhere. GRIND folded into ANAEROBIC. Jump work lives in the POWER SYSTEM only (ruling 4).</x:t>
-        </x:is>
+      <x:c r="A77" s="3" t="str">
+        <x:v>5. NO SLEDS anywhere. GRIND folded into ANAEROBIC. Jump work lives in the POWER SYSTEM only (ruling 4).</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
-      <x:c r="A78" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">6. MID-SESSION MIXING — FLUSH-ONLY PROPERTY (ruling 5). On the three Flush Intervals rows the athlete may rotate machines and/or running BETWEEN ROUNDS within one session. This is the only place in the sheet where a single session spans modalities; everywhere else one session renders on one modality.</x:t>
-        </x:is>
+      <x:c r="A78" s="3" t="str">
+        <x:v>6. MID-SESSION MIXING — FLUSH-ONLY PROPERTY (ruling 5). On the three Flush Intervals rows the athlete may rotate machines and/or running BETWEEN ROUNDS within one session. This is the only place in the sheet where a single session spans modalities; everywhere else one session renders on one modality.</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
-      <x:c r="A79" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">7. INTENSITY CLASSIFIES, W:R IS ONLY A PROPERTY (Sam, V3-final) — see the law at the top of this tab. Do not re-file a session because its ratio sits outside a band, and do not re-dose it to fit one.</x:t>
-        </x:is>
+      <x:c r="A79" s="3" t="str">
+        <x:v>7. INTENSITY CLASSIFIES, W:R IS ONLY A PROPERTY (Sam, V3-final) — see the law at the top of this tab. Do not re-file a session because its ratio sits outside a band, and do not re-dose it to fit one.</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
-      <x:c r="A80" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
+      <x:c r="A80" s="3"/>
     </x:row>
     <x:row r="81">
-      <x:c r="A81" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">HOW TO READ THE CHANGE MARKS</x:t>
-        </x:is>
+      <x:c r="A81" s="2" t="str">
+        <x:v>HOW TO READ THE CHANGE MARKS</x:v>
       </x:c>
     </x:row>
     <x:row r="82">
-      <x:c r="A82" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">MOVED = re-filed to a different quality tab. MERGED = one or more templates folded in (named). SPLIT = one template became two rows. FRAMEWORK-ALIGNED = dose replaced by the framework's numbers. SCHEMA-FILLED = a missing work/rest/set value supplied. NEW = added by a V3 ruling. CONFIRMED = a V2 draft Sam has now signed off. The Change Log tab traces all 99 V2-base rows plus the V3 additions.</x:t>
-        </x:is>
+      <x:c r="A82" s="3" t="str">
+        <x:v>MOVED = re-filed to a different quality tab. MERGED = one or more templates folded in (named). SPLIT = one template became two rows. FRAMEWORK-ALIGNED = dose replaced by the framework's numbers. SCHEMA-FILLED = a missing work/rest/set value supplied. NEW = added by a V3 ruling. CONFIRMED = a V2 draft Sam has now signed off. The Change Log tab traces all 99 V2-base rows plus the V3 additions.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6262,6 +6114,132 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="4.889999866485596" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="30" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="30" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="30" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="30" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="30" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="15" hidden="0" customHeight="1">
+      <x:c r="A1" s="14" t="str">
+        <x:v>Session</x:v>
+      </x:c>
+      <x:c r="B1" s="14" t="str">
+        <x:v>Order</x:v>
+      </x:c>
+      <x:c r="C1" s="14" t="str">
+        <x:v>Section</x:v>
+      </x:c>
+      <x:c r="D1" s="14" t="str">
+        <x:v>Work</x:v>
+      </x:c>
+      <x:c r="E1" s="14" t="str">
+        <x:v>Recovery</x:v>
+      </x:c>
+      <x:c r="F1" s="14" t="str">
+        <x:v>Amount</x:v>
+      </x:c>
+      <x:c r="G1" s="14" t="str">
+        <x:v>Effort</x:v>
+      </x:c>
+      <x:c r="H1" s="14" t="str">
+        <x:v>Cue</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2" s="16" t="str">
+        <x:v>Change of Direction</x:v>
+      </x:c>
+      <x:c r="B2" s="16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C2" s="16" t="str">
+        <x:v>Low-Intensity Deceleration Drills</x:v>
+      </x:c>
+      <x:c r="D2" s="16" t="str">
+        <x:v>20 m build-up + 3 m controlled stop</x:v>
+      </x:c>
+      <x:c r="E2" s="16" t="str">
+        <x:v>Start every 30 s</x:v>
+      </x:c>
+      <x:c r="F2" s="16" t="str">
+        <x:v>10 reps</x:v>
+      </x:c>
+      <x:c r="G2" s="16" t="str">
+        <x:v>4/10</x:v>
+      </x:c>
+      <x:c r="H2" s="16" t="str">
+        <x:v>Lower your body and stop under control.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
+      <x:c r="A3" s="16" t="str">
+        <x:v>Change of Direction</x:v>
+      </x:c>
+      <x:c r="B3" s="16" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C3" s="16" t="str">
+        <x:v>45-Degree Cut Reps</x:v>
+      </x:c>
+      <x:c r="D3" s="16" t="str">
+        <x:v>10 m approach + cut + 10 m exit</x:v>
+      </x:c>
+      <x:c r="E3" s="16" t="str">
+        <x:v>Start every 60 s</x:v>
+      </x:c>
+      <x:c r="F3" s="16" t="str">
+        <x:v>5 reps per side</x:v>
+      </x:c>
+      <x:c r="G3" s="16" t="str">
+        <x:v>10/10</x:v>
+      </x:c>
+      <x:c r="H3" s="16" t="str">
+        <x:v>Keep your plant foot underneath you.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="16" t="str">
+        <x:v>Change of Direction</x:v>
+      </x:c>
+      <x:c r="B4" s="16" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C4" s="16" t="str">
+        <x:v>Up-Back Shuttle</x:v>
+      </x:c>
+      <x:c r="D4" s="16" t="str">
+        <x:v>30 m out + 30 m back</x:v>
+      </x:c>
+      <x:c r="E4" s="16" t="str">
+        <x:v>Start every 60 s</x:v>
+      </x:c>
+      <x:c r="F4" s="16" t="str">
+        <x:v>15 reps</x:v>
+      </x:c>
+      <x:c r="G4" s="16" t="str">
+        <x:v>7/10</x:v>
+      </x:c>
+      <x:c r="H4" s="16" t="str">
+        <x:v>Plant cleanly and accelerate out of the turn.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R467acec2e7684f4f"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -6379,7 +6357,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="5" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C5" s="5" t="n">
         <x:v>0</x:v>
@@ -6489,7 +6467,7 @@
         </x:is>
       </x:c>
       <x:c r="B10" s="6" t="n">
-        <x:v>55</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C10" s="6" t="n">
         <x:v>0</x:v>
@@ -6542,10 +6520,8 @@
           <x:t xml:space="preserve">Previous sheet</x:t>
         </x:is>
       </x:c>
-      <x:c r="B13" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">99 templates (+4 row-level EMPTY notes, deleted) — now 55 rows</x:t>
-        </x:is>
+      <x:c r="B13" s="5" t="str">
+        <x:v>99 templates (+4 row-level EMPTY notes, deleted) — now 52 rows</x:v>
       </x:c>
       <x:c r="C13" s="5" t="inlineStr">
         <x:is>
@@ -6574,10 +6550,8 @@
           <x:t xml:space="preserve">Inferred count</x:t>
         </x:is>
       </x:c>
-      <x:c r="B14" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">was 51 of 99; now 0 of 55 (the framework supplied real doses for the rest)</x:t>
-        </x:is>
+      <x:c r="B14" s="5" t="str">
+        <x:v>was 51 of 99; now 0 of 52 (the framework supplied real doses for the rest)</x:v>
       </x:c>
       <x:c r="C14" s="5" t="inlineStr">
         <x:is>
@@ -8203,304 +8177,102 @@
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Up-Back Shuttle</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B2" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">kept · FINAL ruling 5: availability gate applied</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C2" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">≈11 s (30 m out, 180° turn, 30 m back)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D2" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">≈30–40 s walk</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E2" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">15–20 reps inside 10–15 min</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F2" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Hard but controlled — turn quality is the governor</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G2" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">≈1:3</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H2" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">10–15 min after warm-up</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I2" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No framework band — COD/Decel is not a row in Sam's governing table (mechanics quality). W:R shown for information only. Dose APPROVED AS DRAFTED by Sam's FINAL ruling 5.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J2" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">AVAILABILITY GATE: prescribe only in weeks with NO team training (late off-season, Christmas break) · LOW selection priority</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K2" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Turn should be sharp and controlled, not a slide — plant and go.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L2" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">distance</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M2" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Run-only (field sprint/cutting mechanics; rule 4). No machine rendering.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N2" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Bible Sect.7 L1627–1632 / L606–611 (the only structured COD example the Bible gives); rest, reps, W:R computed in v2</x:t>
-        </x:is>
+      <x:c r="A2" s="5" t="str">
+        <x:v>Change of Direction</x:v>
+      </x:c>
+      <x:c r="B2" s="7" t="str">
+        <x:v>COMBINED 2026-09-02 — one selectable COD session with three ordered sections.</x:v>
+      </x:c>
+      <x:c r="C2" s="5" t="str">
+        <x:v>Three ordered running sections</x:v>
+      </x:c>
+      <x:c r="D2" s="5" t="str">
+        <x:v>As prescribed in each section</x:v>
+      </x:c>
+      <x:c r="E2" s="5" t="str">
+        <x:v>3 sections</x:v>
+      </x:c>
+      <x:c r="F2" s="5" t="str">
+        <x:v>4–10/10</x:v>
+      </x:c>
+      <x:c r="G2" s="5" t="str">
+        <x:v>Varies by section</x:v>
+      </x:c>
+      <x:c r="H2" s="5" t="str">
+        <x:v>≈40 min including warm-up</x:v>
+      </x:c>
+      <x:c r="I2" s="5" t="str">
+        <x:v>No framework band — one occasional ordered mechanics session, not a separately trained energy-system quality.</x:v>
+      </x:c>
+      <x:c r="J2" s="5" t="str">
+        <x:v>AVAILABILITY GATE: prescribe only in weeks with NO team training (late off-season, Christmas break) · LOW selection priority</x:v>
+      </x:c>
+      <x:c r="K2" s="5" t="str">
+        <x:v>Control the stop first, then build into sharper cuts and turns.</x:v>
+      </x:c>
+      <x:c r="L2" s="5" t="str">
+        <x:v>reps</x:v>
+      </x:c>
+      <x:c r="M2" s="5" t="str">
+        <x:v>Run-only (field sprint/cutting mechanics; rule 4). No machine rendering.</x:v>
+      </x:c>
+      <x:c r="N2" s="5" t="str">
+        <x:v>Sam ruling 2026-09-02: combine the three retained COD drills into one ordered session and remove Deceleration and Landing Work.</x:v>
       </x:c>
       <x:c r="O2" s="10" t="str">
         <x:v>run</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Low-Intensity Deceleration Drills</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B3" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">kept · FINAL ruling 5: dose approved as drafted; availability gate applied</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C3" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">≈5 s (jog in, controlled stop over 15–20 m)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D3" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">30–45 s walk-back</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E3" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2–4 reps</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F3" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Low intensity — braking under control</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G3" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">≈1:8</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H3" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">≈3–5 min</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I3" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No framework band — COD/Decel is not a row in Sam's governing table (mechanics quality). W:R shown for information only. Dose APPROVED AS DRAFTED by Sam's FINAL ruling 5.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J3" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">AVAILABILITY GATE: prescribe only in weeks with NO team training (late off-season, Christmas break) · LOW selection priority</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K3" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">This is about braking under control, not stopping like you hit a wall.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L3" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">distance</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M3" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Run-only (field sprint/cutting mechanics; rule 4). No machine rendering.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N3" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Bible names this for building-back athletes (L1758) with no dose; structure drafted here and APPROVED by Sam's FINAL ruling 5</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O3" s="10" t="str">
-        <x:v>run</x:v>
-      </x:c>
+      <x:c r="A3" s="5"/>
+      <x:c r="B3" s="7"/>
+      <x:c r="C3" s="5"/>
+      <x:c r="D3" s="5"/>
+      <x:c r="E3" s="5"/>
+      <x:c r="F3" s="5"/>
+      <x:c r="G3" s="5"/>
+      <x:c r="H3" s="5"/>
+      <x:c r="I3" s="5"/>
+      <x:c r="J3" s="5"/>
+      <x:c r="K3" s="5"/>
+      <x:c r="L3" s="5"/>
+      <x:c r="M3" s="5"/>
+      <x:c r="N3" s="5"/>
+      <x:c r="O3" s="10"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Deceleration and Landing Work</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B4" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">kept (V3-final ruling 3) · FINAL ruling 5: dose approved as drafted; availability gate applied</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C4" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">3–5 s per rep (jump-land-stick / run-and-stick)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D4" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">45–60 s</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E4" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">3–4 reps</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F4" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Controlled landings, quiet feet — quality-gated</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G4" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">≈1:12</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H4" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">≈4–5 min</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I4" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No framework band — COD/Decel is not a row in Sam's governing table (mechanics quality). W:R shown for information only. Dose APPROVED AS DRAFTED by Sam's FINAL ruling 5. STAYS IN COD per Sam's V3-final ruling 3: landing MECHANICS, not jump training (the deleted repeated-jumps session was jump training).</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J4" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">AVAILABILITY GATE: prescribe only in weeks with NO team training (late off-season, Christmas break) · LOW selection priority</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K4" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Stick the landing — quiet feet, not a crash.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L4" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">reps</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M4" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Run-only (field sprint/cutting mechanics; rule 4). No machine rendering.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N4" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Bible names this (L1739) with no dose; structure drafted here and APPROVED by Sam's FINAL ruling 5</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O4" s="10" t="str">
-        <x:v>run</x:v>
-      </x:c>
+      <x:c r="A4" s="5"/>
+      <x:c r="B4" s="7"/>
+      <x:c r="C4" s="5"/>
+      <x:c r="D4" s="5"/>
+      <x:c r="E4" s="5"/>
+      <x:c r="F4" s="5"/>
+      <x:c r="G4" s="5"/>
+      <x:c r="H4" s="5"/>
+      <x:c r="I4" s="5"/>
+      <x:c r="J4" s="5"/>
+      <x:c r="K4" s="5"/>
+      <x:c r="L4" s="5"/>
+      <x:c r="M4" s="5"/>
+      <x:c r="N4" s="5"/>
+      <x:c r="O4" s="10"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">45-Degree Cut Reps</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B5" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">kept · FINAL ruling 5: dose approved as drafted; availability gate applied</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C5" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">≈4 s (10 m in / cut / 10 m out)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D5" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">60–90 s (full recovery)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E5" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">4–6 reps</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F5" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Maximal-intent cut, mechanics-gated</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G5" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">≈1:20</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H5" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">≈5–9 min</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I5" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No framework band — COD/Decel is not a row in Sam's governing table (mechanics quality). W:R shown for information only. Dose APPROVED AS DRAFTED by Sam's FINAL ruling 5.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J5" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">AVAILABILITY GATE: prescribe only in weeks with NO team training (late off-season, Christmas break) · LOW selection priority</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K5" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Plant foot stays under you — if the knee caves, stop the session.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L5" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">distance</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M5" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Run-only (field sprint/cutting mechanics; rule 4). No machine rendering.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N5" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Standard COD drill, not in the Bible; dose drafted here and APPROVED by Sam's FINAL ruling 5</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O5" s="10" t="str">
-        <x:v>run</x:v>
-      </x:c>
+      <x:c r="A5" s="5"/>
+      <x:c r="B5" s="7"/>
+      <x:c r="C5" s="5"/>
+      <x:c r="D5" s="5"/>
+      <x:c r="E5" s="5"/>
+      <x:c r="F5" s="5"/>
+      <x:c r="G5" s="5"/>
+      <x:c r="H5" s="5"/>
+      <x:c r="I5" s="5"/>
+      <x:c r="J5" s="5"/>
+      <x:c r="K5" s="5"/>
+      <x:c r="L5" s="5"/>
+      <x:c r="M5" s="5"/>
+      <x:c r="N5" s="5"/>
+      <x:c r="O5" s="10"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>